<commit_message>
Lab 2: sample files with books instead of bikes
</commit_message>
<xml_diff>
--- a/erp_exchange/samples/export_with_errors.xlsx
+++ b/erp_exchange/samples/export_with_errors.xlsx
@@ -446,16 +446,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DXTR1000</t>
+          <t>BOOK1001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MTB</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1200</v>
+        <v>9.99</v>
       </c>
       <c r="E2" t="n">
         <v>25</v>
@@ -464,12 +464,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GRVL1000</t>
+          <t>BOOK1002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gravel</t>
+          <t>The Hobbit</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -484,12 +484,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ROAD2000</t>
+          <t>BOOK2001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Road Bike</t>
+          <t>Dune</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -502,16 +502,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CITY1000</t>
+          <t>BOOK3001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>City Bike</t>
+          <t>Brave New World</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>499</v>
+        <v>10.99</v>
       </c>
       <c r="E5" t="n">
         <v>2.5</v>
@@ -520,16 +520,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>KIDS1000</t>
+          <t>BOOK3002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kids Bike</t>
+          <t>The Little Prince</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>199</v>
+        <v>7.99</v>
       </c>
       <c r="E6" t="n">
         <v>-1</v>
@@ -538,11 +538,11 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>No ID Bike</t>
+          <t>Book without ID</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>99</v>
+        <v>9.99</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
@@ -551,11 +551,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EBIK1000</t>
+          <t>BOOK3003</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2999</v>
+        <v>11.99</v>
       </c>
       <c r="E8" t="n">
         <v>4</v>
@@ -564,16 +564,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DXTR1000</t>
+          <t>BOOK1001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MTB duplicate</t>
+          <t>1984 (duplicate)</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1150</v>
+        <v>9.49</v>
       </c>
       <c r="E9" t="n">
         <v>20</v>
@@ -582,17 +582,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TREK1000</t>
+          <t>BOOK2002</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Trekking</t>
+          <t>Pride and Prejudice</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>899,90</t>
+          <t>7,90</t>
         </is>
       </c>
       <c r="E10" t="n">

</xml_diff>

<commit_message>
Lab 2 fixes: product form stock/erp_id, keep descriptions, link duplicates, ISBN covers, stay on page, upload log, README
</commit_message>
<xml_diff>
--- a/erp_exchange/samples/export_with_errors.xlsx
+++ b/erp_exchange/samples/export_with_errors.xlsx
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BOOK1001</t>
+          <t>9780451524935</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -464,7 +464,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BOOK1002</t>
+          <t>9780547928227</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -484,7 +484,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BOOK2001</t>
+          <t>9780441172719</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -502,7 +502,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BOOK3001</t>
+          <t>9780060850524</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -520,7 +520,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BOOK3002</t>
+          <t>9780156012195</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -551,7 +551,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BOOK3003</t>
+          <t>9780743273565</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -564,7 +564,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BOOK1001</t>
+          <t>9780451524935</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -582,7 +582,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BOOK2002</t>
+          <t>9780141439518</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">

</xml_diff>